<commit_message>
docs(sistemas): Excel enfocado a Sección 2 — pendientes de 9 a 4, + densidades y silos 5/6
Por confirmar queda solo con lo que bloquea Línea 1 Sección 2: nombres
completos de los 4 tags 066_C (silos 5/6), unidad de F_SL_FlakeFlow_PV,
polaridad de OK_BOMBAS y el alcance del silo de polvo 8. Lo del tramo de
preparación queda en MAPEO-WINCC.md para cuando se cablee.

Tags nuevos: F_CL/F_SL_FlakeDens_PV (la densidad se mide en las dosing bins
y aplica a los silos 5/6) y los 4 de nivel/descarga de silos 5 y 6 con la
advertencia kg/h→kg/min.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
+++ b/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Por confirmar" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$56</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$62</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="242">
   <si>
     <t xml:space="preserve">NOVOPAN · Línea 1 — Tags del HMI para el simulador de trazabilidad</t>
   </si>
@@ -435,6 +435,27 @@
     <t xml:space="preserve">CONFIRMAR POLARIDAD (igual que el anterior).</t>
   </si>
   <si>
+    <t xml:space="preserve">F_CL_FlakeDens_PV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Densidad de flakes en la dosificadora gruesa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg/m³</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se usa como densidad del silo 5 (core): el bin se llena directo del silo con el mismo material.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F_SL_FlakeDens_PV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Densidad de flakes en la dosificadora fina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se usa como densidad del silo 6 (capa fina).</t>
+  </si>
+  <si>
     <t xml:space="preserve">F_CL_FlakeFlow_PV</t>
   </si>
   <si>
@@ -474,6 +495,39 @@
     <t xml:space="preserve">datos/hmi-preparacion.csv</t>
   </si>
   <si>
+    <t xml:space="preserve">066_C_Dry_Materia… (¿?)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCRN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silo 5 (capa interna · core) — nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE INCOMPLETO: clic en el tag y leer la barra de estado abajo del diálogo. Comment: "Nivel silo capa interna %". Alimenta Sección 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silo 5 (capa interna · core) — descarga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg/h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE INCOMPLETO (ídem). Comment: "Descarga desde silo capa interna kg/h". OJO: el simulador lo usa en kg/min — mandar el valor crudo en kg/h, nosotros convertimos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silo 6 (capa externa · fina) — nivel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE INCOMPLETO (ídem). Comment: "Nivel silo capa externa %". Alimenta Sección 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silo 6 (capa externa · fina) — descarga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOMBRE INCOMPLETO (ídem). Comment: "Descarga desde silo capa externa kg/h". Mandar crudo en kg/h.</t>
+  </si>
+  <si>
     <t xml:space="preserve">051_S_Saw_Dust_Level</t>
   </si>
   <si>
@@ -495,9 +549,6 @@
     <t xml:space="preserve">Silo aserrín — densidad</t>
   </si>
   <si>
-    <t xml:space="preserve">kg/m³</t>
-  </si>
-  <si>
     <t xml:space="preserve">051_S_Saw_Dust_Cap</t>
   </si>
   <si>
@@ -666,25 +717,13 @@
     <t xml:space="preserve">Nombre incompleto</t>
   </si>
   <si>
-    <t xml:space="preserve">Los 4 tags que empiezan con 066_C_Dry_Materia… (Access SCRN). Sus comentarios son "Nivel silo capa interna %", "Descarga desde silo capa interna kg/h", "Nivel silo capa externa %" y "Descarga desde silo capa externa kg/h". Necesitamos el nombre completo de los cuatro.</t>
+    <t xml:space="preserve">Los 4 tags que empiezan con 066_C_Dry_Materia… (Access SCRN). Sus comentarios son "Nivel silo capa interna %", "Descarga desde silo capa interna kg/h", "Nivel silo capa externa %" y "Descarga desde silo capa externa kg/h". Necesitamos el nombre completo de los cuatro (clic en el tag → el nombre completo sale en la barra de estado abajo del diálogo).</t>
   </si>
   <si>
     <t xml:space="preserve">Sistemas</t>
   </si>
   <si>
-    <t xml:space="preserve">Son los silos finales 5 (core) y 6 (capa fina) — los que alimentan Sección 2. Es lo más importante de esta lista.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los 3 tags que empiezan con Wet_Mat_CALC_T… (Access WETB): "Total wet material kg/h to 051.60 dosing bunker", su versión en % y "Total dry material kg/h".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es el flujo de material húmedo que entra al bunker dosificador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">La descarga de cada silo húmedo: los tags de 051_S_Saw_Dust_D…, 051_S_Flakes_2_De… y 051_S_Hombak_De… cuyos comentarios son "desc. kg/h" y "desc. kg/h seco".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cierra el caudal de salida de los tres silos verdes.</t>
+    <t xml:space="preserve">Son los silos 5 (core) y 6 (capa fina) — la entrada de Sección 2. Es lo más importante de esta lista.</t>
   </si>
   <si>
     <t xml:space="preserve">¿En qué unidad está F_SL_FlakeFlow_PV? Su comentario dice solo "SL flake flow".</t>
@@ -693,12 +732,6 @@
     <t xml:space="preserve">Lo estamos usando como kg/min. Si es kg/h, el modelo se equivoca por 60×.</t>
   </si>
   <si>
-    <t xml:space="preserve">¿051_S_*_Cap está en m³ o en kg? ¿051_S_*_Level y 051_D_Bunker_Level están en % o en volumen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definen el tiempo que el material pasa dentro de cada silo.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Polaridad</t>
   </si>
   <si>
@@ -708,34 +741,13 @@
     <t xml:space="preserve">Al revés, el simulador marcaría la línea parada justo cuando está corriendo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Correspondencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿Los silos que el HMI llama "aserrín", "flakes 1", "flakes 2" y "hombak" son, en el mismo orden, los que en planta se numeran Silo 1, Silo 2A, Silo 2B y Silo 3?</t>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¿El silo que el HMI llama "silo de polvo 8" (nivel_silo8, Access BRNR) alimenta solo al quemador, o también dosifica material a Sección 2?</t>
   </si>
   <si>
     <t xml:space="preserve">Producción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sin este sí no se pueden cablear 31 parámetros del tramo de preparación. Es la pregunta que más desbloquea.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ambigüedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El código de área 041.11 aparece a la vez como "TSF SILO3" y como "OLD_DATA Sawdust". ¿Es el silo 3 el que transporta aserrín, o el número se reusa para otra cosa?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sistemas / Producción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Determina de qué silo sale el material del secador 1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿El silo que el HMI llama "silo de polvo 8" (nivel_silo8, Access BRNR) alimenta solo al quemador, o también dosifica material a Sección 2?</t>
   </si>
   <si>
     <t xml:space="preserve">En el modelo hay un "Silo 8" que dosifica a Sección 2. Creemos que NO son el mismo.</t>
@@ -1575,7 +1587,7 @@
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTA(Tags!C2:C100)</f>
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1584,7 +1596,7 @@
       </c>
       <c r="C36" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"1 · Crítico")</f>
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1611,7 +1623,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">COUNTA('Por confirmar'!B2:B40)</f>
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,7 +1647,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
@@ -2370,7 +2382,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
         <v>113</v>
       </c>
@@ -2387,13 +2399,13 @@
         <v>137</v>
       </c>
       <c r="F30" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="G30" s="20" t="s">
-        <v>91</v>
+        <v>138</v>
+      </c>
+      <c r="G30" s="24" t="s">
+        <v>55</v>
       </c>
       <c r="H30" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2404,21 +2416,23 @@
         <v>114</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D31" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F31" s="20" t="s">
-        <v>141</v>
-      </c>
-      <c r="G31" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H31" s="22"/>
+        <v>138</v>
+      </c>
+      <c r="G31" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
@@ -2428,23 +2442,25 @@
         <v>114</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D32" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F32" s="20" t="s">
-        <v>141</v>
+        <v>63</v>
       </c>
       <c r="G32" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="H32" s="22"/>
-    </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H32" s="22" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
         <v>113</v>
       </c>
@@ -2452,314 +2468,316 @@
         <v>114</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="F33" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="G33" s="20"/>
-      <c r="H33" s="25" t="s">
-        <v>146</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="F33" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="G33" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H33" s="22"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="B34" s="26" t="s">
+      <c r="A34" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="F34" s="20" t="s">
         <v>148</v>
       </c>
-      <c r="C34" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E34" s="28" t="s">
+      <c r="G34" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H34" s="22"/>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C35" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="F34" s="23" t="s">
+      <c r="D35" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="E35" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="G34" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H34" s="25" t="s">
+      <c r="F35" s="23" t="s">
+        <v>148</v>
+      </c>
+      <c r="G35" s="20"/>
+      <c r="H35" s="25" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="B35" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C35" s="27" t="s">
+    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="D35" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E35" s="28" t="s">
+      <c r="B36" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="F35" s="26" t="s">
+      <c r="C36" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="G35" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H35" s="28"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="B36" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C36" s="27" t="s">
+      <c r="D36" s="26" t="s">
         <v>157</v>
-      </c>
-      <c r="D36" s="26" t="s">
-        <v>150</v>
       </c>
       <c r="E36" s="28" t="s">
         <v>158</v>
       </c>
-      <c r="F36" s="23" t="s">
-        <v>159</v>
+      <c r="F36" s="26" t="s">
+        <v>67</v>
       </c>
       <c r="G36" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H36" s="25" t="s">
+      <c r="H36" s="28" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="E37" s="28" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="B37" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="C37" s="27" t="s">
+      <c r="F37" s="26" t="s">
         <v>161</v>
-      </c>
-      <c r="D37" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E37" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="F37" s="23" t="s">
-        <v>152</v>
       </c>
       <c r="G37" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H37" s="25"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H37" s="28" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C38" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D38" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="E38" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="D38" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E38" s="28" t="s">
-        <v>164</v>
-      </c>
-      <c r="F38" s="23" t="s">
-        <v>152</v>
+      <c r="F38" s="26" t="s">
+        <v>67</v>
       </c>
       <c r="G38" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H38" s="25"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H38" s="28" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B39" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C39" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="D39" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="E39" s="28" t="s">
         <v>165</v>
       </c>
-      <c r="D39" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E39" s="28" t="s">
-        <v>166</v>
-      </c>
       <c r="F39" s="26" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="G39" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H39" s="28"/>
+      <c r="H39" s="28" t="s">
+        <v>166</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B40" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C40" s="27" t="s">
         <v>167</v>
       </c>
       <c r="D40" s="26" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E40" s="28" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F40" s="23" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="G40" s="29" t="s">
         <v>55</v>
       </c>
       <c r="H40" s="25" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C41" s="27" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E41" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="F41" s="23" t="s">
-        <v>152</v>
+        <v>173</v>
+      </c>
+      <c r="F41" s="26" t="s">
+        <v>138</v>
       </c>
       <c r="G41" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H41" s="25"/>
+      <c r="H41" s="28"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C42" s="27" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D42" s="26" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E42" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="F42" s="26" t="s">
-        <v>156</v>
+        <v>175</v>
+      </c>
+      <c r="F42" s="23" t="s">
+        <v>176</v>
       </c>
       <c r="G42" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H42" s="28"/>
+      <c r="H42" s="25" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C43" s="27" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D43" s="26" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E43" s="28" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F43" s="23" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="G43" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H43" s="25" t="s">
-        <v>160</v>
-      </c>
+      <c r="H43" s="25"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C44" s="27" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D44" s="26" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E44" s="28" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="F44" s="23" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="G44" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="H44" s="25" t="s">
-        <v>178</v>
-      </c>
+      <c r="H44" s="25"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B45" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C45" s="27" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D45" s="26" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E45" s="28" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F45" s="26" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="G45" s="29" t="s">
         <v>55</v>
@@ -2768,190 +2786,196 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B46" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C46" s="27" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D46" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="E46" s="28" t="s">
+        <v>185</v>
+      </c>
+      <c r="F46" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="E46" s="28" t="s">
-        <v>182</v>
-      </c>
-      <c r="F46" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="G46" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H46" s="28"/>
+      <c r="G46" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H46" s="25" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B47" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C47" s="27" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D47" s="26" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E47" s="28" t="s">
-        <v>184</v>
-      </c>
-      <c r="F47" s="26" t="s">
-        <v>141</v>
-      </c>
-      <c r="G47" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H47" s="28"/>
+        <v>187</v>
+      </c>
+      <c r="F47" s="23" t="s">
+        <v>170</v>
+      </c>
+      <c r="G47" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H47" s="25"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B48" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C48" s="27" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D48" s="26" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="E48" s="28" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F48" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G48" s="26" t="s">
-        <v>70</v>
+        <v>138</v>
+      </c>
+      <c r="G48" s="29" t="s">
+        <v>55</v>
       </c>
       <c r="H48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B49" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C49" s="27" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D49" s="26" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E49" s="28" t="s">
-        <v>188</v>
-      </c>
-      <c r="F49" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G49" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H49" s="28"/>
+        <v>191</v>
+      </c>
+      <c r="F49" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="G49" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H49" s="25" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C50" s="27" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="D50" s="26" t="s">
-        <v>150</v>
+        <v>193</v>
       </c>
       <c r="E50" s="28" t="s">
-        <v>190</v>
-      </c>
-      <c r="F50" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G50" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H50" s="28"/>
+        <v>194</v>
+      </c>
+      <c r="F50" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="G50" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H50" s="25" t="s">
+        <v>195</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B51" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C51" s="27" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D51" s="26" t="s">
-        <v>150</v>
+        <v>193</v>
       </c>
       <c r="E51" s="28" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="F51" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G51" s="26" t="s">
-        <v>91</v>
+        <v>122</v>
+      </c>
+      <c r="G51" s="29" t="s">
+        <v>55</v>
       </c>
       <c r="H51" s="28"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B52" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C52" s="27" t="s">
+        <v>198</v>
+      </c>
+      <c r="D52" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="E52" s="28" t="s">
+        <v>199</v>
+      </c>
+      <c r="F52" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="C52" s="27" t="s">
-        <v>193</v>
-      </c>
-      <c r="D52" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="E52" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="F52" s="26" t="s">
-        <v>141</v>
-      </c>
       <c r="G52" s="26" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="H52" s="28"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B53" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" s="27" t="s">
+        <v>200</v>
+      </c>
+      <c r="D53" s="26" t="s">
+        <v>193</v>
+      </c>
+      <c r="E53" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="F53" s="26" t="s">
         <v>148</v>
-      </c>
-      <c r="C53" s="27" t="s">
-        <v>195</v>
-      </c>
-      <c r="D53" s="26" t="s">
-        <v>196</v>
-      </c>
-      <c r="E53" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="F53" s="26" t="s">
-        <v>67</v>
       </c>
       <c r="G53" s="26" t="s">
         <v>70</v>
@@ -2960,22 +2984,22 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B54" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C54" s="27" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="D54" s="26" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="E54" s="28" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F54" s="26" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="G54" s="26" t="s">
         <v>70</v>
@@ -2984,19 +3008,19 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B55" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C55" s="27" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D55" s="26" t="s">
-        <v>196</v>
+        <v>168</v>
       </c>
       <c r="E55" s="28" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F55" s="26" t="s">
         <v>67</v>
@@ -3006,34 +3030,178 @@
       </c>
       <c r="H55" s="28"/>
     </row>
-    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="26" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B56" s="26" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C56" s="27" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D56" s="26" t="s">
-        <v>204</v>
+        <v>168</v>
       </c>
       <c r="E56" s="28" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F56" s="26" t="s">
-        <v>206</v>
+        <v>67</v>
       </c>
       <c r="G56" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="H56" s="28" t="s">
-        <v>207</v>
+      <c r="H56" s="28"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B57" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C57" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="D57" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="E57" s="28" t="s">
+        <v>209</v>
+      </c>
+      <c r="F57" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="G57" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H57" s="28"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B58" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C58" s="27" t="s">
+        <v>210</v>
+      </c>
+      <c r="D58" s="26" t="s">
+        <v>168</v>
+      </c>
+      <c r="E58" s="28" t="s">
+        <v>211</v>
+      </c>
+      <c r="F58" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="G58" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H58" s="28"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B59" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C59" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="D59" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="E59" s="28" t="s">
+        <v>214</v>
+      </c>
+      <c r="F59" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="G59" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H59" s="28"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B60" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C60" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="D60" s="26" t="s">
+        <v>216</v>
+      </c>
+      <c r="E60" s="28" t="s">
+        <v>217</v>
+      </c>
+      <c r="F60" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G60" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H60" s="28"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B61" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C61" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="D61" s="26" t="s">
+        <v>213</v>
+      </c>
+      <c r="E61" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="F61" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="G61" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H61" s="28"/>
+    </row>
+    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B62" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="C62" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="D62" s="26" t="s">
+        <v>221</v>
+      </c>
+      <c r="E62" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="F62" s="26" t="s">
+        <v>223</v>
+      </c>
+      <c r="G62" s="26" t="s">
+        <v>91</v>
+      </c>
+      <c r="H62" s="28" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H62"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3050,7 +3218,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -3061,142 +3229,72 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>215</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="30" t="s">
-        <v>212</v>
+        <v>46</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>216</v>
+        <v>233</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>217</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>214</v>
+        <v>231</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="30" t="s">
-        <v>46</v>
+        <v>238</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>220</v>
+        <v>239</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>214</v>
+        <v>240</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>222</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="30" t="s">
-        <v>224</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>225</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>214</v>
-      </c>
-      <c r="D7" s="18" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="B8" s="25" t="s">
-        <v>228</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="30" t="s">
-        <v>231</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>232</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>233</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
-        <v>235</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>236</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: Excel solo-Sección-2 (39 tags, 3 pendientes) + plan del adaptador de formatos CSV
El Excel deja únicamente el tramo silos 5/6 → sensores para que Sistemas
responda rápido; el upstream queda en MAPEO-WINCC.md para una segunda tanda.
El plan del adaptador define sniffer → perfil (kv/tabla/ancho) → normalizador
al formato canónico, con calidad de dato y fixtures antes de codificar.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
+++ b/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Por confirmar" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$40</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="184">
   <si>
     <t xml:space="preserve">NOVOPAN · Línea 1 — Tags del HMI para el simulador de trazabilidad</t>
   </si>
@@ -528,178 +528,16 @@
     <t xml:space="preserve">NOMBRE INCOMPLETO (ídem). Comment: "Descarga desde silo capa externa kg/h". Mandar crudo en kg/h.</t>
   </si>
   <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WETS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% ⚠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">⚠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD: ¿m³ o kg?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_1_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 1 — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — nivel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Dens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — densidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Cap</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_D_Bunker_Level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WETB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — nivel calculado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR UNIDAD: ¿% o m³?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_3_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — peso (900A1.3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_1_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — caudal 1 (900A1.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_A1_2_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — caudal 2 (900A1.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_60_B1_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bunker dosificador — humedad (902T2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Saw_Dust_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo aserrín — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Flakes_2_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_S_Hombak_Hum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo hombak — humedad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">051_08_SL7_OUTxEU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Silo flakes 2 — transmisor de nivel (897T4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">071_DRY_Hum_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRYR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Humedad a la salida del secadero</t>
-  </si>
-  <si>
     <t xml:space="preserve">Prensa_metal_detector</t>
   </si>
   <si>
     <t xml:space="preserve">Prensa</t>
   </si>
   <si>
-    <t xml:space="preserve">Metal detectado en el material</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimiento_sec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimiento del secadero</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta_T_out</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Memory)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delta T entrada – salida del tambor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">°C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es Memory Real del HMI: puede no existir en el PLC. Si no sale, se omite.</t>
+    <t xml:space="preserve">Metal detectado en el material (detector a 37.69 m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Está en el servidor de Preparación aunque el equipo es de Sección 2.</t>
   </si>
   <si>
     <t xml:space="preserve">Tema</t>
@@ -739,18 +577,6 @@
   </si>
   <si>
     <t xml:space="preserve">Al revés, el simulador marcaría la línea parada justo cuando está corriendo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¿El silo que el HMI llama "silo de polvo 8" (nivel_silo8, Access BRNR) alimenta solo al quemador, o también dosifica material a Sección 2?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Producción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En el modelo hay un "Silo 8" que dosifica a Sección 2. Creemos que NO son el mismo.</t>
   </si>
 </sst>
 </file>
@@ -1587,7 +1413,7 @@
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTA(Tags!C2:C100)</f>
-        <v>61</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1596,7 +1422,7 @@
       </c>
       <c r="C36" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"1 · Crítico")</f>
-        <v>25</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1605,7 +1431,7 @@
       </c>
       <c r="C37" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"2 · Deseado")</f>
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1614,7 +1440,7 @@
       </c>
       <c r="C38" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"3 · Opcional")</f>
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1623,7 +1449,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">COUNTA('Por confirmar'!B2:B40)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1647,7 +1473,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
@@ -2636,7 +2462,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="26" t="s">
         <v>154</v>
       </c>
@@ -2652,556 +2478,18 @@
       <c r="E40" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="F40" s="23" t="s">
+      <c r="F40" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G40" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H40" s="28" t="s">
         <v>170</v>
       </c>
-      <c r="G40" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H40" s="25" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B41" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C41" s="27" t="s">
-        <v>172</v>
-      </c>
-      <c r="D41" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E41" s="28" t="s">
-        <v>173</v>
-      </c>
-      <c r="F41" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G41" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H41" s="28"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B42" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C42" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="D42" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E42" s="28" t="s">
-        <v>175</v>
-      </c>
-      <c r="F42" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G42" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H42" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B43" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C43" s="27" t="s">
-        <v>178</v>
-      </c>
-      <c r="D43" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E43" s="28" t="s">
-        <v>179</v>
-      </c>
-      <c r="F43" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G43" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H43" s="25"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B44" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C44" s="27" t="s">
-        <v>180</v>
-      </c>
-      <c r="D44" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E44" s="28" t="s">
-        <v>181</v>
-      </c>
-      <c r="F44" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G44" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H44" s="25"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B45" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C45" s="27" t="s">
-        <v>182</v>
-      </c>
-      <c r="D45" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E45" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="F45" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G45" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H45" s="28"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B46" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C46" s="27" t="s">
-        <v>184</v>
-      </c>
-      <c r="D46" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E46" s="28" t="s">
-        <v>185</v>
-      </c>
-      <c r="F46" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G46" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H46" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B47" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C47" s="27" t="s">
-        <v>186</v>
-      </c>
-      <c r="D47" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E47" s="28" t="s">
-        <v>187</v>
-      </c>
-      <c r="F47" s="23" t="s">
-        <v>170</v>
-      </c>
-      <c r="G47" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H47" s="25"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B48" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C48" s="27" t="s">
-        <v>188</v>
-      </c>
-      <c r="D48" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E48" s="28" t="s">
-        <v>189</v>
-      </c>
-      <c r="F48" s="26" t="s">
-        <v>138</v>
-      </c>
-      <c r="G48" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H48" s="28"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B49" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C49" s="27" t="s">
-        <v>190</v>
-      </c>
-      <c r="D49" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E49" s="28" t="s">
-        <v>191</v>
-      </c>
-      <c r="F49" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G49" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H49" s="25" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C50" s="27" t="s">
-        <v>192</v>
-      </c>
-      <c r="D50" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E50" s="28" t="s">
-        <v>194</v>
-      </c>
-      <c r="F50" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="G50" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H50" s="25" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B51" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C51" s="27" t="s">
-        <v>196</v>
-      </c>
-      <c r="D51" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E51" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="F51" s="26" t="s">
-        <v>122</v>
-      </c>
-      <c r="G51" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H51" s="28"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B52" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C52" s="27" t="s">
-        <v>198</v>
-      </c>
-      <c r="D52" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E52" s="28" t="s">
-        <v>199</v>
-      </c>
-      <c r="F52" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G52" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H52" s="28"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B53" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C53" s="27" t="s">
-        <v>200</v>
-      </c>
-      <c r="D53" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E53" s="28" t="s">
-        <v>201</v>
-      </c>
-      <c r="F53" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G53" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H53" s="28"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B54" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C54" s="27" t="s">
-        <v>202</v>
-      </c>
-      <c r="D54" s="26" t="s">
-        <v>193</v>
-      </c>
-      <c r="E54" s="28" t="s">
-        <v>203</v>
-      </c>
-      <c r="F54" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G54" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H54" s="28"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B55" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C55" s="27" t="s">
-        <v>204</v>
-      </c>
-      <c r="D55" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E55" s="28" t="s">
-        <v>205</v>
-      </c>
-      <c r="F55" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G55" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H55" s="28"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B56" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C56" s="27" t="s">
-        <v>206</v>
-      </c>
-      <c r="D56" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E56" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="F56" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G56" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H56" s="28"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B57" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C57" s="27" t="s">
-        <v>208</v>
-      </c>
-      <c r="D57" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E57" s="28" t="s">
-        <v>209</v>
-      </c>
-      <c r="F57" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G57" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H57" s="28"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B58" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C58" s="27" t="s">
-        <v>210</v>
-      </c>
-      <c r="D58" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E58" s="28" t="s">
-        <v>211</v>
-      </c>
-      <c r="F58" s="26" t="s">
-        <v>148</v>
-      </c>
-      <c r="G58" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H58" s="28"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B59" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C59" s="27" t="s">
-        <v>212</v>
-      </c>
-      <c r="D59" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="E59" s="28" t="s">
-        <v>214</v>
-      </c>
-      <c r="F59" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G59" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H59" s="28"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B60" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C60" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="D60" s="26" t="s">
-        <v>216</v>
-      </c>
-      <c r="E60" s="28" t="s">
-        <v>217</v>
-      </c>
-      <c r="F60" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="G60" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H60" s="28"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B61" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C61" s="27" t="s">
-        <v>218</v>
-      </c>
-      <c r="D61" s="26" t="s">
-        <v>213</v>
-      </c>
-      <c r="E61" s="28" t="s">
-        <v>219</v>
-      </c>
-      <c r="F61" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G61" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H61" s="28"/>
-    </row>
-    <row r="62" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B62" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C62" s="27" t="s">
-        <v>220</v>
-      </c>
-      <c r="D62" s="26" t="s">
-        <v>221</v>
-      </c>
-      <c r="E62" s="28" t="s">
-        <v>222</v>
-      </c>
-      <c r="F62" s="26" t="s">
-        <v>223</v>
-      </c>
-      <c r="G62" s="26" t="s">
-        <v>91</v>
-      </c>
-      <c r="H62" s="28" t="s">
-        <v>224</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H62"/>
+  <autoFilter ref="A1:H40"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3218,7 +2506,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -3229,30 +2517,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>225</v>
+        <v>171</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>226</v>
+        <v>172</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>227</v>
+        <v>173</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>228</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>229</v>
+        <v>175</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>230</v>
+        <v>176</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>232</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3260,41 +2548,27 @@
         <v>46</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>233</v>
+        <v>179</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>234</v>
+        <v>180</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="30" t="s">
-        <v>235</v>
+        <v>181</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>236</v>
+        <v>182</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>231</v>
+        <v>177</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="30" t="s">
-        <v>238</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>239</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="D5" s="18" t="s">
-        <v>241</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(sistemas): descartar OK_BOMBAS_GLUING — la línea se asume siempre corriendo
Decisión de alcance: una parada se detecta por los flujos y velocidades, que ya
llegan. Pedirlos obligaba a resolver la contradicción entre el nombre ("OK") y
el comentario del HMI ("FALLA"), y costaba más de lo que ahorraba.

Se quitan los dos tags de la hoja Tags, no solo el pendiente de polaridad: si
solo se borraba el pendiente, Sistemas igual iba a ir a buscarlos.

37 tags · 2 pendientes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
+++ b/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Por confirmar" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$40</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Tags!$A$1:$H$38</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="174">
   <si>
     <t xml:space="preserve">NOVOPAN · Línea 1 — Tags del HMI para el simulador de trazabilidad</t>
   </si>
@@ -414,27 +414,6 @@
     <t xml:space="preserve">Nivel de la tolva dosificadora fina</t>
   </si>
   <si>
-    <t xml:space="preserve">OK_BOMBAS_GLUING_CL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bombas de encolado grueso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0/1 ⚠</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR POLARIDAD: el nombre dice OK pero el comentario dice "FALLA BOMBAS ENCOLADO CL".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK_BOMBAS_GLUING_SL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bombas de encolado fino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CONFIRMAR POLARIDAD (igual que el anterior).</t>
-  </si>
-  <si>
     <t xml:space="preserve">F_CL_FlakeDens_PV</t>
   </si>
   <si>
@@ -568,15 +547,6 @@
   </si>
   <si>
     <t xml:space="preserve">Lo estamos usando como kg/min. Si es kg/h, el modelo se equivoca por 60×.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polaridad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OK_BOMBAS_GLUING_CL y _SL: ¿1 significa que están OK, o que hay falla? El nombre dice una cosa y el comentario del HMI dice la contraria.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Al revés, el simulador marcaría la línea parada justo cuando está corriendo.</t>
   </si>
 </sst>
 </file>
@@ -1413,7 +1383,7 @@
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTA(Tags!C2:C100)</f>
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1431,7 +1401,7 @@
       </c>
       <c r="C37" s="13" t="n">
         <f aca="false">COUNTIF(Tags!G2:G100,"2 · Deseado")</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1449,7 +1419,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">COUNTA('Por confirmar'!B2:B40)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1473,7 +1443,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
@@ -2172,13 +2142,13 @@
       <c r="E28" s="22" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="23" t="s">
+      <c r="F28" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="G28" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H28" s="25" t="s">
+      <c r="G28" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="H28" s="22" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2198,17 +2168,17 @@
       <c r="E29" s="22" t="s">
         <v>134</v>
       </c>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="G29" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="H29" s="25" t="s">
+      <c r="G29" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="H29" s="22" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="20" t="s">
         <v>113</v>
       </c>
@@ -2225,13 +2195,13 @@
         <v>137</v>
       </c>
       <c r="F30" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" s="22" t="s">
         <v>138</v>
-      </c>
-      <c r="G30" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="H30" s="22" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2242,23 +2212,21 @@
         <v>114</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D31" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E31" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="F31" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="F31" s="20" t="s">
-        <v>138</v>
-      </c>
-      <c r="G31" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="H31" s="22" t="s">
-        <v>142</v>
-      </c>
+      <c r="G31" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H31" s="22"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
@@ -2268,25 +2236,23 @@
         <v>114</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D32" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F32" s="20" t="s">
-        <v>63</v>
+        <v>141</v>
       </c>
       <c r="G32" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="H32" s="22" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H32" s="22"/>
+    </row>
+    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
         <v>113</v>
       </c>
@@ -2294,85 +2260,89 @@
         <v>114</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D33" s="20" t="s">
         <v>116</v>
       </c>
       <c r="E33" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="F33" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="G33" s="20"/>
+      <c r="H33" s="25" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="26" t="s">
         <v>147</v>
       </c>
-      <c r="F33" s="20" t="s">
+      <c r="B34" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G33" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H33" s="22"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="C34" s="21" t="s">
+      <c r="C34" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="D34" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="E34" s="22" t="s">
+      <c r="D34" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="F34" s="20" t="s">
+      <c r="E34" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="F34" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="G34" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H34" s="28" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B35" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G34" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="H34" s="22"/>
-    </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20" t="s">
-        <v>113</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>114</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>151</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>116</v>
-      </c>
-      <c r="E35" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="F35" s="23" t="s">
+      <c r="C35" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="D35" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E35" s="28" t="s">
+        <v>153</v>
+      </c>
+      <c r="F35" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="G35" s="29" t="s">
+        <v>55</v>
+      </c>
+      <c r="H35" s="28" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B36" s="26" t="s">
         <v>148</v>
       </c>
-      <c r="G35" s="20"/>
-      <c r="H35" s="25" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B36" s="26" t="s">
-        <v>155</v>
-      </c>
       <c r="C36" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="D36" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E36" s="28" t="s">
         <v>156</v>
-      </c>
-      <c r="D36" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="E36" s="28" t="s">
-        <v>158</v>
       </c>
       <c r="F36" s="26" t="s">
         <v>67</v>
@@ -2381,115 +2351,63 @@
         <v>55</v>
       </c>
       <c r="H36" s="28" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="B37" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="D37" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="E37" s="28" t="s">
+        <v>158</v>
+      </c>
+      <c r="F37" s="26" t="s">
         <v>154</v>
-      </c>
-      <c r="B37" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C37" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="D37" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="E37" s="28" t="s">
-        <v>160</v>
-      </c>
-      <c r="F37" s="26" t="s">
-        <v>161</v>
       </c>
       <c r="G37" s="29" t="s">
         <v>55</v>
       </c>
       <c r="H37" s="28" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="26" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="B38" s="26" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="C38" s="27" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="E38" s="28" t="s">
+        <v>162</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>74</v>
+      </c>
+      <c r="G38" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="H38" s="28" t="s">
         <v>163</v>
       </c>
-      <c r="F38" s="26" t="s">
-        <v>67</v>
-      </c>
-      <c r="G38" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H38" s="28" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B39" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C39" s="27" t="s">
-        <v>156</v>
-      </c>
-      <c r="D39" s="26" t="s">
-        <v>157</v>
-      </c>
-      <c r="E39" s="28" t="s">
-        <v>165</v>
-      </c>
-      <c r="F39" s="26" t="s">
-        <v>161</v>
-      </c>
-      <c r="G39" s="29" t="s">
-        <v>55</v>
-      </c>
-      <c r="H39" s="28" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="26" t="s">
-        <v>154</v>
-      </c>
-      <c r="B40" s="26" t="s">
-        <v>155</v>
-      </c>
-      <c r="C40" s="27" t="s">
-        <v>167</v>
-      </c>
-      <c r="D40" s="26" t="s">
-        <v>168</v>
-      </c>
-      <c r="E40" s="28" t="s">
-        <v>169</v>
-      </c>
-      <c r="F40" s="26" t="s">
-        <v>74</v>
-      </c>
-      <c r="G40" s="26" t="s">
-        <v>70</v>
-      </c>
-      <c r="H40" s="28" t="s">
-        <v>170</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H40"/>
+  <autoFilter ref="A1:H38"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2506,7 +2424,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -2517,30 +2435,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B2" s="25" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D2" s="18" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2548,27 +2466,13 @@
         <v>46</v>
       </c>
       <c r="B3" s="25" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="D3" s="18" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
-        <v>181</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>182</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>177</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
decision(hmi-csv): F_SL_FlakeFlow_PV se asume kg/min — 0 pendientes
El comentario del HMI no declara unidad. Se fija kg/min por simetría con su
gemelo H_CL_Total_Flakes ("CL total flakes kg/min") y con los tags hermanos
del grupo SL_DosBin, que sí la declaran.

Queda anotado en el código cómo revertirlo si el dato en vivo lo desmiente:
si el valor sale ~60x fuera de H_CL_Total_Flakes, era kg/h y basta cambiar el
alias a { tag: 'F_SL_KGMIN', scale: 1/60 }.

El Excel para Sistemas queda en 37 tags y 0 pendientes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
+++ b/parte-2-aglomerados/deck/simulador-final/NOVOPAN_L1_Tags_HMI_para_Sistemas.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="172">
   <si>
     <t xml:space="preserve">NOVOPAN · Línea 1 — Tags del HMI para el simulador de trazabilidad</t>
   </si>
@@ -540,13 +540,7 @@
     <t xml:space="preserve">Por qué importa</t>
   </si>
   <si>
-    <t xml:space="preserve">¿En qué unidad está F_SL_FlakeFlow_PV? Su comentario dice solo "SL flake flow".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sistemas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lo estamos usando como kg/min. Si es kg/h, el modelo se equivoca por 60×.</t>
+    <t xml:space="preserve">Nada pendiente. Todos los tags de esta lista están confirmados y listos para volcar — ver la hoja «Tags».</t>
   </si>
 </sst>
 </file>
@@ -556,7 +550,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -682,6 +676,14 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1B5E20"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -897,8 +899,8 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1419,7 +1421,7 @@
       </c>
       <c r="C39" s="13" t="n">
         <f aca="false">COUNTA('Por confirmar'!B2:B40)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2447,21 +2449,18 @@
         <v>170</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="30" t="s">
-        <v>46</v>
-      </c>
-      <c r="B2" s="25" t="s">
         <v>171</v>
       </c>
-      <c r="C2" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>173</v>
-      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>